<commit_message>
feat: nuevo Usos_Espec 24 familias, fix carrito hidden marker, fix buscarEnUsos scoring
</commit_message>
<xml_diff>
--- a/data/cruzeiro/Usos_Especificaciones.xlsx
+++ b/data/cruzeiro/Usos_Especificaciones.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30131"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://cruzeiroempresas-my.sharepoint.com/personal/jcornejo_cruzeiroempresas_cl/Documents/Escritorio/Cruzeiro Gomas JC/Proyecto BOT-CRM/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{81A90C8C-7FE2-4EFA-A943-D09C2FC4688E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="171" documentId="8_{81A90C8C-7FE2-4EFA-A943-D09C2FC4688E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{28F7F984-D07E-41A5-AED0-C6BA0567AF62}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="20730" windowHeight="11040" xr2:uid="{A1BA93E0-6444-4574-9298-686B45B2876E}"/>
   </bookViews>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="333" uniqueCount="300">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="379" uniqueCount="340">
   <si>
     <t>PISOS GOMA EN ROLLO SIN TELA</t>
   </si>
@@ -3791,34 +3791,6 @@
 Una de sus mayores ventajas técnicas en el mercado chileno es su fórmula segura: no contiene solventes prohibidos ni altamente tóxicos como tolueno, benceno o compuestos clorados, lo que facilita su aplicación segura en interiores ventilados.</t>
   </si>
   <si>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="12"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>Usos y Aplicaciones Principales</t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Calibri"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve">
-Instalación de Revestimientos y Pisos: Es el estándar para fijar rollos de goma, pisos de caucho, vinilos, alfombras y palmetas de pasto sintético sobre bases de concreto o madera.
-Industria del Caucho y Goma: Se emplea masivamente para pegar planchas de goma (como EVA, neopreno o SBR) y perfiles técnicos en canales metálicos.
-Tapicería y Automoción: Ideal para el pegado de espumas, telas, cueros y revestimientos internos en la restauración de asientos de vehículos, techos de cabinas y paneles de puertas.
-Mueblería y Carpintería: Utilizado para el laminado de Formalita (laminados plásticos) sobre tableros de madera, MDF o aglomerados.
-Calzado y Marroquinería: Reparación y armado de calzado mediante la unión firme de suelas de goma con cuero o materiales sintéticos.</t>
-    </r>
-  </si>
-  <si>
     <t>Especificaciones Técnicas y Rendimiento
 Rendimiento: Rinde aproximadamente entre 4 y 5 metros cuadrados por litro por capa.
 Tiempo de secado para contacto: Requiere dejar evaporar los solventes entre 15 y 30 minutos antes de unir las piezas.Temperatura de trabajo: Se recomienda aplicar en ambientes entre 10°C y 35°C.
@@ -3870,6 +3842,505 @@
 Cierres herméticos de compuertas pesadas: Actúa como junta de estanqueidad en compuertas de descarga de silos, tolvas de áridos, mezcladoras de hormigón y portones industriales que ejercen un fuerte cierre por pernos o palancas.
 Topes e insertos antivibración: Funciona como barra o pasador amortiguador en uniones mecánicas, bases de maquinaria pesada y soportes estructurales para disipar ráfagas de vibración y evitar el choque directo metal-metal.
 Juntas de dilatación pesadas en construcción: Se inserta a presión como cordón de relleno estructural en juntas de expansión profundas de pisos industriales de concreto antes de aplicar el sellador elastomérico final.</t>
+  </si>
+  <si>
+    <t>CONTENEDOR DE BASURA</t>
+  </si>
+  <si>
+    <t>Uso por Colores (Reciclaje Seguro)</t>
+  </si>
+  <si>
+    <t>Contenedor Azul: Cartón, papeles, diarios, revistas y cajas de embalaje limpias.
+Contenedor Amarillo: Envases plásticos, botellas de PET, latas de aluminio y envases de Tetra Pak.
+Contenedor Verde: Botellas de vidrio, frascos y tarros sin tapas metálicas ni plásticas.
+Contenedor Gris o Negro: Residuos comunes, basura orgánica residencial y desechos no reciclables.
+Contenedor Café: Desechos orgánicos puros, restos de comida, cáscaras y residuos de jardinería.</t>
+  </si>
+  <si>
+    <t>Uso por Capacidad y Diseño</t>
+  </si>
+  <si>
+    <t>Los contenedores de basura se clasifican principalmente por su color de reciclaje, capacidad en litros y material de fabricación HDPE para garantizar una correcta gestión de los residuos.
+En Cruzeiro comercializamos de Plástico polietileno (HDPE): Soportan golpes, climas extremos, rayos UV y son fáciles de lavar.</t>
+  </si>
+  <si>
+    <t>De 10 a 50 litros: Uso interior en cocinas, oficinas, baños y habitaciones pequeñas.
+De 120 a 240 litros: Uso residencial exterior, equipados con ruedas para facilitar la recolección municipal.
+De 660 a 1100 litros: Uso comunitario, edificios, condominios, industrias y zonas comerciales de alto tráfico.</t>
+  </si>
+  <si>
+    <t>Uso en Interior de la Casa</t>
+  </si>
+  <si>
+    <t>Cocina (20 a 30 Litros): Requiere mecanismos que eviten usar las manos, como los basureros con pedal o tapas basculantes, y materiales fáciles de limpiar como el acero inoxidable o plástico reforzado.
+Módulos de Reciclaje (Apilables): Ideales si cuentas con poco espacio en la cocina o logia, ya que permiten clasificar residuos de forma vertical sin obstruir el paso.
+Baños y Dormitorios (5 a 12 Litros): Basureros pequeños, generalmente con pedal, que quepan fácilmente en rincones o bajo los muebles.</t>
+  </si>
+  <si>
+    <t>Uso para Exterior/Jardín</t>
+  </si>
+  <si>
+    <t>Requisitos Clave para Exteriores
+Material HDPE: Deben ser de Polietileno de Alta Densidad para soportar impactos pesados, químicos y cambios de temperatura extremas sin agrietarse.
+Hermeticidad y Control: Tapas de calce preciso que eviten el ingreso de agua de lluvia, impidan que entren vectores (perros, roedores, insectos) y contengan los malos olores.
+Norma EN840: Si se saca el contenedor a la calle, contar con esta certificación asegura que sus pestañas frontales resistan los brazos hidráulicos de los camiones recolectores municipales en Chile.</t>
+  </si>
+  <si>
+    <t>Para cubrir tanto el hogar como la oficina, las soluciones de limpieza y celulosa se dividen en formatos domésticos (enfocados en el cuidado de superficies delicadas y comodidad) e institucionales (diseñados para alta rotación, dosificación eficiente y máxima higiene).</t>
+  </si>
+  <si>
+    <t>Productos de Papel y Celulosa</t>
+  </si>
+  <si>
+    <t>Papel Higiénico Tradicional vs. Jumbo:
+Hogar: Rollos estándar de 30 a 50 metros (hoja doble o triple) que priorizan la suavidad al tacto.
+Oficina: Rollos industriales Jumbo de 200 a 400 metros para dispensadores cerrados, reduciendo la frecuencia de reposición y evitando hurtos.
+Opciones: Papel Higiénico Elite Jumbo Doble Hoja de 250 metros (Ideal para baños de empresas) o Papel Higiénico Confort 50 metros Doble Hoja (Para el hogar).
+Toallas de Papel (Secado de Manos y Superficies):
+Hogar: Rollos de cocina absorbentes para derrames o frituras.
+Oficina: Toallas de papel interfoliadas (en formato Z o C) para dispensadores de pared en baños y cocinas comunitarias, asegurando que el usuario solo toque la hoja que va a usar.
+Opciones: Toalla Interfoliada Elite Extra Blanco Dispensador
+Pañuelos y Servilletas:
+Uso: Servilletas para comedores/casinos y pañuelos desechables en cajas (tissues) para escritorios y salas de reuniones.</t>
+  </si>
+  <si>
+    <t>Productos de Aseo Químico</t>
+  </si>
+  <si>
+    <t>Desinfectantes de Superficies y Pisos:
+Hogar: Limpiadores líquidos aromatizados (lavanda, contratipo de cloro) para una desinfección suave y diaria de pisos cerámicos y flotantes.
+Oficina: Desinfectantes concentrados a base de Amonio Cuaternario para eliminar patógenos en áreas de alto tránsito (recepciones, pasillos y baños) sin dañar los pisos de alto tráfico.
+Opciones: Amonio Cuaternario Concentrado (Formato industrial de 5 litros) o Limpiador Líquido Multiuso.
+Higienizantes de Contacto Directo (Escritorios y Tecnología):
+Hogar: Toallitas húmedas comunes para mesones.
+Oficina: Alcohol isopropílico en aerosol, toallitas desinfectantes y amonios listos para usar. Son indispensables para limpiar teclados, ratones, pantallas, teléfonos fijos y cubiertas de escritorios compartidos.
+Opciones: Toallitas Desinfectantes (Eliminan virus en superficies de oficina) o Limpia Equipos Electrónicos Perfumerías Unidas.
+Jabón e Higiene de Manos:
+Hogar: Jabón líquido en botella con dosificador recargable.
+Oficina: Jabón líquido o en espuma para dispensadores empotrados, generalmente en cartuchos sellados de 800 ml o 1 litro que garantizan que el producto no se contamine.
+Especialidades (Limpiavidrios y Lustramuebles):
+Uso: El limpiavidrios es crucial en oficinas con ventanales o mamparas divisorias para eliminar huellas dactilares. El lustramuebles protege escritorios de melamina o madera.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Lavado de Ropa (Detergentes de Alto Rendimiento)
+Lavado de Vajilla y Desengrasantes
+Limpieza y Desinfección de Pisos
+Sanitización Profunda (Baños y Cocinas)
+Betún de Zapatos
+Bolsas de Basura
+Cera para auto
+Cloro
+Cloro Gel
+Desodorante Ambiental
+Desorante WC
+Esponja cocina
+Lavaloza
+Limpiador en Crema
+Mopa
+Respuesto Mopa
+</t>
+  </si>
+  <si>
+    <t>Otros Productos Aseo</t>
+  </si>
+  <si>
+    <t>ASEO Y PRODUCTOS PAPEL, HOGAR Y OFICINA.
+CLEANHAUS</t>
+  </si>
+  <si>
+    <t>PRODUCTOS DECORACIÓN.
+DECOHAUS</t>
+  </si>
+  <si>
+    <t>Las categorías de Decoración (Deco) y diseño de interiores se clasifican según la función que cumplen en los espacios y el impacto visual o sensorial que generan.</t>
+  </si>
+  <si>
+    <t>Los accesorios de organización para baños se diseñan con materiales resistentes a la humedad (como acero inoxidable, plástico acrílico y cerámica) para optimizar los metros cuadrados en zonas críticas como la ducha, el vanitorio y los muebles inferiores.
+Organizadores para Ducha y TinaAprovechan la altura de los muros para mantener los champús, geles y esponjas al alcance, evitando que los productos queden acumulados en el suelo o los bordes de la tina:
+BL NH 2 GANCHOS SUCCIÓN BLANCA 4112NH
+BL NH 3 GANCHOS CUADRADOS PEQUEÑOS ACERO INOXIDABLE 1313NH
+BL NH 4 GANCHOS DE LUJO 0758NH
+BL NH ATRAPA PELOS 0871NH
+BL NH CANASTO ESQUINERO SUCCION 4009NH
+BL NH ESQUINERO SUCCION BLANCA 4109NH
+BL NH PERCHA 3 GANCHOS SUCCIÓN BLANCA 4123NH
+BL NH PORTA ROLLO STANDARD 0850NH
+BL NH REPUESTO PARA PORTA ROLLO 0853NH
+BL NH SUJETADOR MULTIUSO TRIPLE SUCCIÓN FUERTE 4129NH
+NH CANASTO MULTIUSO SUCCION CROMADO 4206NH
+NH CANASTO SUCCION CROMADA 4208NH
+NH CINTA DE SELLADO IMPERMEABLE 4.1 CMS. MULTIUSO
+NH COLGADOR CROMADO FALDA/PANTALONES C/CLI 0557NH
+NH COLGADOR MADERA C/CLIPS 0981NH
+NH COLGADOR MADERA MULTIUSO 0971NH
+NH ORGANIZADOR DUCHA GRANDE CON PORTA JABÓN PLÁSTICO 0118NH
+NH ORGANIZADOR PARA DUCHA 0116NH
+NH REPISA SUCCION CROMADA 4210NH
+NH SECAPL/SECAV CROM/PLAST/NEGRO 2506NH
+NH SECAPLATOS CON SECAVASOS CROMADO 1506NH
+SET BAÑO 14 PIEZAS SIDNEY</t>
+  </si>
+  <si>
+    <t>Productos Organización Baños</t>
+  </si>
+  <si>
+    <t>Productos Organización Cocina</t>
+  </si>
+  <si>
+    <t>Los artículos de decoración para la cocina se caracterizan por combinar estética y funcionalidad ("decoración útil"), empleando materiales duraderos y fáciles de limpiar (como madera tratada, vidrio, cerámica y metal) para transformar la encimera y las paredes sin entorpecer las labores culinarias:
+BATERIA DE COCINA 460-8SS  CACEROLAS 18 - 24 - 26 -CAZO 16 CMS.
+BOTELLA VIDRIO FUNDA COLOR 525 CC
+CONTENEDOR HERMETICO VIDRIO CUADRADO 320ML
+CONTENEDOR HERMETICO VIDRIO CUADRADO 380ML
+CONTENEDOR HERMETICO VIDRIO CUADRADO 520ML
+CONTENEDOR HERMETICO VIDRIO CUADRADO 740ML
+CONTENEDOR HERMETICO VIDRIO CUADRADO 800ML
+CONTENEDOR HERMETICO VIDRIO RECT. 1,500 ML
+CONTENEDOR HERMETICO VIDRIO RECT. 1000ML
+CONTENEDOR HERMETICO VIDRIO RECT. 420ML
+CONTENEDOR HERMETICO VIDRIO RECT. 600ML
+CONTENEDOR HERMETICO VIDRIO RECT. 750ML
+CONTENEDOR HERMETICO VIDRIO RECTANGULAR 1040ML
+CONTENEDOR HERMETICO VIDRIO RECTANGULAR 370ML
+CONTENEDOR HERMETICO VIDRIO RECTANGULAR 650ML
+CONTENEDOR HERMETICO VIDRIO REDONDO 370ML
+CONTENEDOR HERMETICO VIDRIO REDONDO 720ML
+CONTENEDOR VIDRIO HERMETICO CUAD. 1200ML GLASSLOCK
+CONTENEDOR VIDRIO HERMETICO CUAD. 490ML GLASSLOCK
+CONTENEDOR VIDRIO HERMETICO RECT. 2000ML GLASSLOCK
+CONTENEDOR VIDRIO HERMETICO RECT. 400ML GLASSLOCK
+CUCHILLO DE AFICION DE PRECISION
+CUCHILLO DE USO
+DESPENSERO REAL GRANDE 3 NIVELES BLANCO OPTICO
+JARRA MEDIDORA 0.5 LTS ALLEGRA
+JARRA MEDIDORA 1.0 LTS ALLEGRA
+JARRA REFRIGERADOR RIVOLI 1,1lts C/TAPA COLOR
+JUEGO DE 10 CUCHILLAS 61MMX19XX WADFOW
+MATAMOSCAS
+SET 3 PAÑOS DE COCINA MICROFIBRA
+SET CUCHILLERÍA COPPER 24 PIEZAS KRONS
+SET DE CUCHILLERÍA 24 PIEZAS GOLD KRONS
+TAPA MICROONDAS 25X25X6
+TERMO MAGNUM STEEL COMIDA ACERO 0,5L
+TERMO MAGNUM STEEL COMIDA ACERO 0,75L
+TERMO NEW MAGNUM COM 0.43 LT. LISO
+TERMO VEW MAGNUM COM 0,75LT. LISO</t>
+  </si>
+  <si>
+    <t>Productos de Dormitorio</t>
+  </si>
+  <si>
+    <t>Los artículos de decoración para el dormitorio están pensados para construir un santuario de descanso, priorizando texturas suaves que absorban el ruido, luces cálidas indirectas y elementos visuales que aporten calma y reflejen tu estilo personal:
+CALIENTA CAMA 1 PLAZA POLIESTER OZU
+MAGEFESA CALIENTACAMA DOMO 2 PLAZAS
+MANTA TERMICA Magefesa Igloo Mgf1580
+OZU CINTURÓN CALEFACTOR ELECTRICO</t>
+  </si>
+  <si>
+    <t>Productos Decoración Jardín</t>
+  </si>
+  <si>
+    <t>Los artículos de decoración para el jardín y patio están diseñados con materiales altamente resistentes a la intemperie (rayos UV, lluvia y viento) para transformar las zonas exteriores en espacios acogedores, dinámicos y llenos de vida tanto de día como de noche.
+COMPOSTERA TORRE 300 L
+MACETA RATAN 25X25X25 CM. C/SIST RIEGO MARRON
+MACETA RATAN 30X30X30 CM. C/SIST RIEGO MARRON
+MACETA RATAN 40X40X40 CM. C/SIST RIEGO MARRON
+MACETA BAMBU COLGANTE GRANDE VERDE
+MACETA DURA KOTTA REDONDA #10 DIAMETRO 28 CM TERRACOTA
+MACETA DURA KOTTA REDONDA #14 DIAMETRO 40CM TERRACOTA
+MACETA REDONDA ESTILO PIEDRA 18 X 16 CM TAUPE
+MACETA REDONDA ESTILO PIEDRA 25X23 CM TAUPE
+MACETA REDONDA ESTILO PIEDRA 33X30 CM TAUPE
+MACETA REDONDA ESTILO RATÁN 18 X 16 CM MARRON MORO
+MACETA REDONDA ESTILO RATÁN 25 X 23 CM MARRON MORO
+MACETA REDONDA ESTILO RATÁN 33 X 30 CM MARRON MORO
+MACETERO SIENA 14 CM, ARENA
+MACETERO SIENA 14 CM, TAUPE
+MACETERO SIENA 20 CM, ARENA
+MACETERO SIENA 20 CM, TAUPE
+MACETERO SIENA 30 CM,ARENA
+MACETERO SIENA 30 CM,TAUPE
+MACETERO SIENA 40 CM TAUPE CON RUEDAS
+MACETERO SIENA 40 CM,ARENA CON RUEDAS
+PLATO DE MACETA RECTANGULAR DURA KOTTA 44CM / TERRACOTA
+PLATO DE MACETA RECTANGULAR DURA KOTTA 44CM / VERDE
+PLATO DE MACETA RECTANGULAR DURA KOTTA 59CM / TERRACOTA
+PLATO DE MACETA RECTANGULAR DURA KOTTA 59CM / VERDE
+PLATO DURA KOTTA REDONDA #10 DIAMETRO 25CM TERRACOTA
+PLATO DURA KOTTA REDONDA #10 DIAMETRO 25CM VERDE
+PLATO DURA KOTTA REDONDA #14 DIAMETRO 35CM TERRACOTA
+PLATO DURA KOTTA REDONDA #14 DIAMETRO 35CM VERDE
+PLATO DURA KOTTA REDONDA #16 DIAMETRO 40CM TERRACOTA
+PLATO DURA KOTTA REDONDA #16 DIAMETRO 40CM VERDE
+PLATO MACETA REDONDA ESTILO  PIEDRA 33X30 CM TAUPE
+PLATO MACETA REDONDA ESTILO PIEDRA  25X 23 CM TAUPE
+PLATO MACETA REDONDA ESTILO RATÁN 18 X 16 CM MARRON MORO
+PLATO MACETA REDONDA ESTILO RATÁN 25 X 23 CM MARRON MORO
+PLATO MACETA REDONDA ESTILO RATÁN 33 X 30 CM MARRON MORO
+PLATO TAZON PARA MASCOTAS METALICO FORRADO 34 CM COLORES VERDE, CAFÉ
+SET CONTENEDOR RECICLAJE 4 COLORES
+SET DE RIEGO Y ACOPLE PARA MANGUERA 1/2</t>
+  </si>
+  <si>
+    <t>Productos Organización Espacios</t>
+  </si>
+  <si>
+    <t>Productos para Parrillas</t>
+  </si>
+  <si>
+    <t>Los productos para parrillas abarcan desde herramientas de cocción hasta insumos de mantenimiento, permitiendo optimizar el encendido, proteger la estructura y lograr asados perfectos.A continuación, se presentan las categorías esenciales de artículos parrilleros disponibles para su compra en Cruzeiro:
+ASADERA CUADRADA 1,8LTS
+ASADERA OPAL OVAL MEDIANA 28,8*17CMS/1,0 LTS
+ASADERA OPAL REDONDA GRANDE 28 CMS/2LT
+ASADERA REC C/ASA 2.7L. SELETTA
+ASADERA REC C/ASA 3.5L. SELETTA
+ASADERA RECTANGULAR GRANDE 2,9LTS
+ASADERA RECTANGULAR MEDIANA 2,2LTS
+ASADERA RECTANGULAR PEQ. 1,6LTS
+CUCHILLA  JUMBO A. INOX. M/MADERA
+CUCHILLO  PARA  PESCADO  8" A.INOX. M/ MADERA
+CUCHILLO  PARA ASADO A INOX. M/MADERA
+CUCHILLO PARA  CARNICERIA  10"
+DISPLAY 6 VASOS ALTOS MIKONOS FONDO COLOR 460 CC
+DISPLAY 6 VASOS ALTOS MONTERREY FONDO COLOR 445 CC
+DISPLAY 6 VASOS ATLANTA 258CC (CRISTAR) 0455CL6STM
+DISPLAY 6 VASOS W/A MIKONOS FULL COLOR  460 CC
+ESPATULA  LARGA CURVA A. INOX. M /POLIPROP
+ESPATULA  LARGA RECTA A. INOX. M /POLIPROP
+JARRA PITCHER 1600ML
+JUEGO  PARA  ASADO 02 PZA A. INOX.M/MADERA
+JUEGO  PARA  ASADO 04 PZA A. INOX.M/MADERA
+PARRILLA   MULTIUSO
+PARRILLA  ARGENTINA  PEQUEÑA
+PARRILLA  COM TAPA DESMONTABLE
+PARRILLA FOGON PASEO
+PARRILLA RODEO CON TAPA
+SET 1 DECANTADOR CASABLANCA 1,7 LTS
+SET 2 CERVECEROS BAVARIA 600 CC
+SET 2 CERVECEROS ZIEL 600CC
+SET 4 CERVECERO AMBERES 560CC
+SET PARRILLERO 2 PIEZAS ACERO INOXIDABLE MANGO DE MADERA. CUCHILLO + TRINCHO
+SET PARRILLERO 3 PZA ACERO INOXIDABLE CON FUNDA 46 CM
+TABLA HERRADURA MADERA 45X25 CM
+TABLA MADERA 35X20 CM
+TENEDOR PARA ASADO A. INOX. M/MADERA
+TENEDOR TRINCHANTE A. INOX M/ MADERA</t>
+  </si>
+  <si>
+    <t>Productos de Temporada</t>
+  </si>
+  <si>
+    <t>Los productos de temporada estival o de verano están diseñados para combatir las altas temperaturas, proteger la salud ante la radiación solar y maximizar el confort en espacios exteriores e interiores:
+BOLSO EMMA CON CORREA DE ALGODON PDQ
+FLOTADOR CISNE NEGRO 45 X 65 CM
+QUITASOL PLAYA 1,8M UV+40
+VENTILADOR DE PEDESTAL 18 GIRO 360°- 5 ASPAS METÁLICAS - 3 VELOCIDADES  (1 UNI)</t>
+  </si>
+  <si>
+    <t>FERRETERÍA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Los artículos de ferretería abarcan las herramientas, fijaciones y equipamientos esenciales utilizados para la construcción, reparación, mantenimiento e instalaciones tanto en el hogar como a nivel profesional:
+ACOPLE RAPIDO  PARA MANGUERA 1/2""
+ACOPLE RAPIDO  PARA MANGUERA 3/4""
+AMARRAS PLASTICAS BLANCA ESP. 4.8 X 350MM (100 UNI)
+AMARRAS PLASTICAS BLANCA ESP. 4.8 X 450MM (100 UNI)
+AMARRAS PLASTICAS NEGRA ESP. 4.8 X 350MM (100 UNI)
+AMARRAS PLASTICAS NEGRA ESP. 4.8 X 380MM (100 UNI)
+AMARRAS PLASTICAS NEGRA ESP. 4.8 X 450MM (100 UNI)
+AMARRAS PLASTICAS NEGRA ESP. 7.2 X 400MM (100 UNI)
+AMARRAS PLASTICAS TRANSP 4.8 X 250MM (100 UNI)
+BALDE CONCRETERO 12LT
+BALDE FLEXIBLE 28 LTS MEZCLA  ADHESIVO
+BATEA RECTANGULAR 100LTS NEGRO
+BATEA REDONDA 50 LTS NEGRO
+BROCHA DE POLIESTER MANGO NATURAL SYD 2 1/2''
+BROCHA MANGO ROJO / CERDAS DE CERDO 5"
+CAJA TALLER AMARILLO
+CAJA TALLER NEGRO
+CINTA METRICA DE ACERO 3MX16 MM
+CINTA METRICA DE ACERO 7,5 MT X 25 MM WADFOW
+CINTA TEFLON BLANCA 1/2" ESP 0.1MM 12MTS
+CINTA TEFLON GAS 1/2" ESP 0.1MM 12MTS
+ESC. ALUMINIO TIJERA 1.52 M.
+ESCALERA ALUMINIO TIJERA 1.83 M.
+ESCUADRA 30X15 CM WADFOW
+ESTANTE  ORGANIZADOR  65X31X154 CM
+GEOTEXTIL BLANCO 200GSM ROLLO 2X75 (DESGLOSE)
+JUEGO DE ALICATES DE 3 PIEZAS (6-6-7") WADFOW
+JUEGO DE DESTORNILLADORES DE 2 PIEZAS 40CR WADFOW
+JUEGO DE PINTURA(RODILLO + BANDEJA)
+LASER DE LINEA AUTONIVENIVELANTE WADFOW
+LAVARROPA 15LTS CON KIT DE INSTALACION
+LAVARROPA 24LTS CON KIT DE INSTALACION
+LLAVE MONOMANDO LAVAMANOS AQUA RAME CARTUCHO 35MM
+LONA MULTIUSO 10X12 M
+LONA MULTIUSO 4X5 M
+MALLA SOMBRA FRANJEADA 80% AZUL Y BLANCO DE 4.20 X 100 MTS.
+MALLA SOMBRA LISA 65% AZUL DE 2.10 X 100 MTS.
+MARTILLO CARPINTERO MANGO DE MADERA 16 OZ
+MAZO DE GOMA BLANCO 450 G
+MONOMANDO DUCHA AQUA RAME CARTUCHO 35MM
+MONOMANDO TINA/DUCHA AQUA RAME CARTUCHO 35MM
+NIVEL ALUMINIO 40 CM
+PERFIL ANGULO PVC 10X10MM BLANCO (T3MT)
+PERFIL ANGULO PVC 32X32MM BLANCO (T3MT)
+PERFIL CUBREJUNTA J ALFOMBRA PVC NE (R50MT)
+PERFIL GUARDAPOLVO RETORNO SANITARIO PVC 50MM BLANCO (T3MT)
+PERFIL SELLO TINA PVC 25X23MM BLANCO (T3MT)
+PERFIL ZOCALO SANITARIO MACHO-HEMBRA SP PVC 100MM BLANCO (T3MT)
+PERFIL ZOCALO SANITARIO MACHO-HEMBRA SP PVC 62MM BLANCO (T3MT)
+PISTOLA DE SILICONA 9" WADFOW
+PLANA CUADRADA 7"" 9.5/180MM
+PLANA LENGÜETA 7"" 7.5/180MM
+PLANCHA AISLAPOL ST 100X50 ESPESOR 40 MM AISLAPOL ,PACK 15 UNIDADES
+PLANCHA AISLAPOL ST 100X50 ESPESOR 50 MM AISLAPOL ,PACK 12 UNIDADES
+REPUESTO CUCHILLA DE 10 HOJAS 18X100 MM
+TALADRO INALAMBRICO 20V+2B+1C WADFOW
+</t>
+  </si>
+  <si>
+    <t>CAJAS AGRO</t>
+  </si>
+  <si>
+    <t>Las cajas agro o cajas agrícolas son contenedores plásticos industriales de alta resistencia diseñados específicamente para optimizar la recolección, el prefrío en cámaras, el transporte y el acopio de hortalizas, frutas y subproductos del campo.Están fabricadas principalmente en Polietileno de Alta Densidad (HDPE) o Polipropileno (PP) de grado alimentario, lo que garantiza su inocuidad y una larga vida útil ante el uso rudo:
+CAJA AGRO BERRIES 45X34 G2 VERDE
+CAJA BULBO WEN PE L2 NEGRO
+CAJA COSECHERA 3/4 RVCG2-L-2</t>
+  </si>
+  <si>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="12"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Usos y Aplicaciones Principales</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">
+Instalación de Revestimientos y Pisos: Es el estándar para fijar rollos de goma, pisos de caucho, vinilos, alfombras y palmetas de pasto sintético sobre bases de concreto o madera.
+Industria del Caucho y Goma: Se emplea masivamente para pegar planchas de goma (como EVA, neopreno o SBR) y perfiles técnicos en canales metálicos.
+Tapicería y Automoción: Ideal para el pegado de espumas, telas, cueros y revestimientos internos en la restauración de asientos de vehículos, techos de cabinas y paneles de puertas como:
+Piso Goma 
+Piso PVC
+Gradas 
+Empaquetaduras
+Piso Nomad
+Piso Gimnasio
+Goma EVA
+Plancha EVA
+Mueblería y Carpintería: Utilizado para el laminado de Formalita (laminados plásticos) sobre tableros de madera, MDF o aglomerados.
+Calzado y Marroquinería: Reparación y armado de calzado mediante la unión firme de suelas de goma con cuero o materiales sintéticos.</t>
+    </r>
+  </si>
+  <si>
+    <t>PRODUCTOS PARA MASCOTAS</t>
+  </si>
+  <si>
+    <t>Los productos de organización de espacios se enfocan en optimizar los metros cuadrados del hogar mediante sistemas verticales, contenedores apilables y divisores internos que reducen el desorden visual y facilitan el acceso diario a los objetos:
+BANCO IDEAL COLORES
+BANCO IDEAL NEGRO
+BANCO ROBLE PLEGABLE GRANDE
+BANCO ROBLE PLEGABLE MEDIANO
+BANQUITO TAVARUA RATAN MARRON CHILE EA
+BASURERO PEDAL CLIN 12,5 LTS METALIZADO
+BASURERO PEDAL DANUBIO 24 LTS BLANCO NEON
+BAUL C/RDA 100L 77X40X48 ROJO/AMARILLO
+BAUL C/RDA 72L 80X40X34 LILA/ROSA
+BAUL C/RDA 72L 80X40X34 VD/AZ
+BAÚL HERRAMIENTAS 73 LTS AMARILLO/NEGRO
+BAUL MEGAFORTE 123 LTS. GRIS/TURQUESA
+BAUL MEGAFORTE 90 LTS AZUL TAPA AZUL
+BAUL MEGAFORTE 90 LTS AZUL TAPA ROJA
+BAUL MEGAFORTE 90 LTS ROJO/NEGRO
+CAJA 100 LTS
+CAJA BAJO CAMA 34L CON RUEDAS
+CAJA BAJO CAMA 48 L CLARIFICADO CELESTE
+CAJA FRONTAL 15 L GRIS CLARIFICADO
+CAJA LUXOR 12 L
+CAJA MEGAFORTE 120 LTS COLORES CHILE
+CAJA MEGAFORTE 38L COLORES
+CAJA MEGAFORTE 75 LTS  COLORES CHILE
+CAJA MULTIUSO MULTIBOX 51 LTS PVV COP BLANCO 60 X 40 AMARILLO
+CAJA ORGANIZADORA 14 LTS
+CAJA SUPREMA 50L CHILE
+CAJA SUPREMA 58 LTS CLARIFICADO
+CAJA SUPREMA 72 LTS CLARIFICADO VERDE
+CAJA ULTRAFORTE FAST MOVIL 210 FOUR SEASONS BEIGE CHOCOLATE
+CAJA VITALBOX 28 LTS C/MANILLA
+CAJA VITALBOX 38 LTS C/MANILLA
+CAJA VITALBOX 66 LTS C/MANILLA
+CANASTA TAVARUA MODELO RATAN MARRON ALMENDRA
+CANASTILLA BOABAB 22L
+CANASTILLA TAVARUA 13 L - BLANCO C/T
+CANASTILLA TAVARUA 13 L - MARRON MORO C/T
+CANASTILLA TAVARUA 22 L - BEIGE HUMO C/T
+CANASTILLA TAVARUA 22 L - BLANCO C/T
+CANASTILLA TAVARUA 22 L - MARRON MORO C/T
+CANASTILLA TAVARUA 5.5 L - TAUPE
+CANASTILLA TAVARUA 6, 5 LT MARRON
+CANASTILLA TAVARUA 6.5 L - MARRON MORO C/T
+CELOSIA PLANA PP 20X20CM BLANCO (U1UN)
+CELOSIA PLANA PP 30X30CM BLANCO (U1UN)
+CESTO KHIPU 40 LTS BEIGE HUMO
+CESTO KHIPU 40LTS GRIS ACERO
+CESTO KHIPU 60 LTS BEIGE
+CESTO KHIPU 60 LTS TAUPE
+CESTO KHIPU 60 LTS. COLORES CHILE
+CESTO MODELO RATAN BALI  CON TAPA MARRON
+CESTO MODELO RATAN GRANDE 62 L CON TAPA MARRON GRANDE
+CESTO MODELO RATAN GRANDE 62L GRIS
+COMODA KUSI RATÁN 3 NIVELES TAPUE
+ESQUINERO CON GAVETERO DE BAÑO BLANCO NEON
+MESA REDONDA CARAL NUEVA  BLANCO
+MESA ROBLE 150X80
+NEVERA 35 LTS ROJO
+NEVERA TAVARUA RATAN 35 LTS MARRÓN MORO
+NH SET 5 COLGADORES 0139NH
+ORGANIZADOR MULTIUSO GRANDE CUERPO COLORES
+PAPELERA MAGALY # 18 METALIZADA
+PAPELERA MAGALY # 30 METALIZADA
+PAPELERO PEDAL 12L
+PAPELERO PEDAL BLANCO 25 LTS. TATAY
+PAPELERO TAPA VAIVEN GRIS 15 LTS.
+REPOSERA CABO BLANCO TAUPE
+REPOSERA CAMASTRO RECLINABLE RESINA CABO BLANCO
+SET CANASTILLA TAVARUA #3
+SET ORGANIZADOR APLILABLE # 15 ROJO
+SET ORGANIZADOR APLILABLE #15 GRIS OSCURO
+SILLA BAR TAVARUA MODELO RATAN MARRON
+SILLA BARCELONA CON BRAZO CHILE
+SILLA MANU -CHILE
+SILLA ROBLE CON BRAZOS
+SILLA ROBLE SIN BRAZO
+SILLA TAVARUA RATAN S/BRAZO MARRON
+TAPA RESPUESTO MEGAFORTE 123 LTS
+TENDEDERO AEREO BUENOS AIRES/2</t>
+  </si>
+  <si>
+    <t>Los productos para mascotas se clasifican según la necesidad biológica o de comportamiento que cubren, abarcando desde la nutrición e higiene básica hasta el enriquecimiento ambiental necesario para perros, gatos y animales exóticos:
+ALFOMBRA PARA DERRAME DE LIQUIDOS CON DISEÑO DE HUESO 63,5X38,1 CM
+ARENA SANITARIA KIBOO PETS NEUTRO 4KG PARA GATO
+COLLAR BUFANDA PARA MASCOTAS CON DISEÑO LARGO HASTA 50 CM
+COLLAR BUFANDA PARA MASCOTAS CON DISEÑO LARGO HASTA 60 CM
+COLLAR KIBOO PETS DE GATO DISEÑO N°1
+COLLAR KIBOO PETS DISEÑO PARA PERRO TL P/PERRO
+COLLAR KIBOO PETS DISEÑO PARA PERRO TM P/PERRO
+COLLAR KIBOO PETS DISEÑO PARA PERRO TS P/PERRO
+COLLAR MASCOTA SIMIL CUERO C/APLICACIONES METALICA LARGO 38CM -COLORES
+SANDWICH KIBOO PETS POLLO Y PESCADO P/GATO
+TABLERO DE RASGUÑO KIBOO PETS N°2 P/GATO</t>
   </si>
 </sst>
 </file>
@@ -3943,7 +4414,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="4">
+  <borders count="6">
     <border>
       <left/>
       <right/>
@@ -3988,11 +4459,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top/>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -4012,15 +4509,10 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
@@ -4030,230 +4522,32 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="35">
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <alignment vertical="top"/>
-    </dxf>
-    <dxf>
-      <fill>
-        <patternFill patternType="solid">
-          <bgColor theme="8" tint="0.59999389629810485"/>
-        </patternFill>
-      </fill>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -4563,10 +4857,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D2DAF943-1E86-4692-AFCD-C08B9BA0554C}">
-  <dimension ref="A1:R66"/>
+  <dimension ref="A1:R79"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="31.5703125" style="13" customWidth="1"/>
+    <col min="1" max="1" width="31.5703125" style="8" customWidth="1"/>
     <col min="2" max="2" width="77.7109375" customWidth="1"/>
     <col min="3" max="3" width="70.5703125" customWidth="1"/>
     <col min="4" max="4" width="68.7109375" customWidth="1"/>
@@ -4587,7 +4881,7 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A1" s="9" t="s">
+      <c r="A1" s="12" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="1" t="s">
@@ -4610,7 +4904,7 @@
       </c>
     </row>
     <row r="2" spans="1:8" ht="90" x14ac:dyDescent="0.25">
-      <c r="A2" s="9"/>
+      <c r="A2" s="12"/>
       <c r="B2" s="3" t="s">
         <v>7</v>
       </c>
@@ -4631,7 +4925,7 @@
       </c>
     </row>
     <row r="3" spans="1:8" ht="105" x14ac:dyDescent="0.25">
-      <c r="A3" s="9"/>
+      <c r="A3" s="12"/>
       <c r="B3" s="3" t="s">
         <v>13</v>
       </c>
@@ -4652,7 +4946,7 @@
       </c>
     </row>
     <row r="4" spans="1:8" ht="90" x14ac:dyDescent="0.25">
-      <c r="A4" s="9"/>
+      <c r="A4" s="12"/>
       <c r="B4" s="3" t="s">
         <v>20</v>
       </c>
@@ -4673,7 +4967,7 @@
       </c>
     </row>
     <row r="5" spans="1:8" ht="75" x14ac:dyDescent="0.25">
-      <c r="A5" s="9"/>
+      <c r="A5" s="12"/>
       <c r="B5" s="3"/>
       <c r="C5" s="3" t="s">
         <v>26</v>
@@ -4685,7 +4979,7 @@
       <c r="F5" s="3"/>
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
-      <c r="A6" s="9" t="s">
+      <c r="A6" s="12" t="s">
         <v>28</v>
       </c>
       <c r="B6" s="1" t="s">
@@ -4708,7 +5002,7 @@
       </c>
     </row>
     <row r="7" spans="1:8" ht="120" x14ac:dyDescent="0.25">
-      <c r="A7" s="9"/>
+      <c r="A7" s="12"/>
       <c r="B7" s="3" t="s">
         <v>36</v>
       </c>
@@ -4729,7 +5023,7 @@
       </c>
     </row>
     <row r="8" spans="1:8" ht="105" x14ac:dyDescent="0.25">
-      <c r="A8" s="9"/>
+      <c r="A8" s="12"/>
       <c r="B8" s="3" t="s">
         <v>43</v>
       </c>
@@ -4750,7 +5044,7 @@
       </c>
     </row>
     <row r="9" spans="1:8" ht="105" x14ac:dyDescent="0.25">
-      <c r="A9" s="9"/>
+      <c r="A9" s="12"/>
       <c r="B9" s="3"/>
       <c r="C9" s="3" t="s">
         <v>49</v>
@@ -4765,7 +5059,7 @@
       <c r="G9" s="3"/>
     </row>
     <row r="10" spans="1:8" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A10" s="10" t="s">
+      <c r="A10" s="9" t="s">
         <v>19</v>
       </c>
       <c r="B10" s="1" t="s">
@@ -4788,7 +5082,7 @@
       </c>
     </row>
     <row r="11" spans="1:8" ht="195.75" x14ac:dyDescent="0.25">
-      <c r="A11" s="10"/>
+      <c r="A11" s="9"/>
       <c r="B11" s="3" t="s">
         <v>58</v>
       </c>
@@ -4809,7 +5103,7 @@
       </c>
     </row>
     <row r="12" spans="1:8" ht="220.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A12" s="10"/>
+      <c r="A12" s="9"/>
       <c r="B12" s="3" t="s">
         <v>65</v>
       </c>
@@ -4830,7 +5124,7 @@
       </c>
     </row>
     <row r="13" spans="1:8" ht="138.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A13" s="10"/>
+      <c r="A13" s="9"/>
       <c r="B13" s="3" t="s">
         <v>71</v>
       </c>
@@ -4845,7 +5139,7 @@
       <c r="G13" s="3"/>
     </row>
     <row r="14" spans="1:8" ht="15" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A14" s="10" t="s">
+      <c r="A14" s="9" t="s">
         <v>74</v>
       </c>
       <c r="B14" s="1" t="s">
@@ -4871,7 +5165,7 @@
       </c>
     </row>
     <row r="15" spans="1:8" ht="182.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A15" s="10"/>
+      <c r="A15" s="9"/>
       <c r="B15" s="3" t="s">
         <v>82</v>
       </c>
@@ -4895,7 +5189,7 @@
       </c>
     </row>
     <row r="16" spans="1:8" ht="120.75" x14ac:dyDescent="0.25">
-      <c r="A16" s="10"/>
+      <c r="A16" s="9"/>
       <c r="B16" s="3" t="s">
         <v>90</v>
       </c>
@@ -4919,7 +5213,7 @@
       </c>
     </row>
     <row r="17" spans="1:7" ht="170.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A17" s="10"/>
+      <c r="A17" s="9"/>
       <c r="C17" s="3" t="s">
         <v>98</v>
       </c>
@@ -4937,7 +5231,7 @@
       </c>
     </row>
     <row r="18" spans="1:7" ht="136.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A18" s="10"/>
+      <c r="A18" s="9"/>
       <c r="C18" s="3" t="s">
         <v>103</v>
       </c>
@@ -4955,7 +5249,7 @@
       </c>
     </row>
     <row r="19" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A19" s="9" t="s">
+      <c r="A19" s="12" t="s">
         <v>35</v>
       </c>
       <c r="B19" s="5" t="s">
@@ -4978,7 +5272,7 @@
       </c>
     </row>
     <row r="20" spans="1:7" ht="189" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A20" s="9"/>
+      <c r="A20" s="12"/>
       <c r="B20" s="3" t="s">
         <v>115</v>
       </c>
@@ -4999,7 +5293,7 @@
       </c>
     </row>
     <row r="21" spans="1:7" ht="210.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A21" s="9"/>
+      <c r="A21" s="12"/>
       <c r="B21" s="3" t="s">
         <v>121</v>
       </c>
@@ -5009,7 +5303,7 @@
       <c r="D21" s="3"/>
     </row>
     <row r="22" spans="1:7" ht="225.75" x14ac:dyDescent="0.25">
-      <c r="A22" s="9"/>
+      <c r="A22" s="12"/>
       <c r="B22" s="3" t="s">
         <v>124</v>
       </c>
@@ -5018,7 +5312,7 @@
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A23" s="9" t="s">
+      <c r="A23" s="12" t="s">
         <v>126</v>
       </c>
       <c r="B23" s="5" t="s">
@@ -5041,7 +5335,7 @@
       </c>
     </row>
     <row r="24" spans="1:7" ht="165" x14ac:dyDescent="0.25">
-      <c r="A24" s="9"/>
+      <c r="A24" s="12"/>
       <c r="B24" s="3" t="s">
         <v>115</v>
       </c>
@@ -5062,7 +5356,7 @@
       </c>
     </row>
     <row r="25" spans="1:7" ht="165.75" x14ac:dyDescent="0.25">
-      <c r="A25" s="9"/>
+      <c r="A25" s="12"/>
       <c r="B25" s="3" t="s">
         <v>121</v>
       </c>
@@ -5072,7 +5366,7 @@
       <c r="D25" s="3"/>
     </row>
     <row r="26" spans="1:7" ht="225.75" x14ac:dyDescent="0.25">
-      <c r="A26" s="9"/>
+      <c r="A26" s="12"/>
       <c r="B26" s="3" t="s">
         <v>124</v>
       </c>
@@ -5081,7 +5375,7 @@
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A27" s="9" t="s">
+      <c r="A27" s="12" t="s">
         <v>42</v>
       </c>
       <c r="B27" s="5" t="s">
@@ -5104,7 +5398,7 @@
       </c>
     </row>
     <row r="28" spans="1:7" ht="188.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A28" s="9"/>
+      <c r="A28" s="12"/>
       <c r="B28" s="3" t="s">
         <v>132</v>
       </c>
@@ -5125,7 +5419,7 @@
       </c>
     </row>
     <row r="29" spans="1:7" ht="270.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A29" s="9"/>
+      <c r="A29" s="12"/>
       <c r="B29" s="3" t="s">
         <v>136</v>
       </c>
@@ -5138,15 +5432,15 @@
       <c r="E29" s="3" t="s">
         <v>138</v>
       </c>
-      <c r="F29" s="7" t="s">
+      <c r="F29" s="13" t="s">
         <v>139</v>
       </c>
-      <c r="G29" s="7" t="s">
+      <c r="G29" s="13" t="s">
         <v>139</v>
       </c>
     </row>
     <row r="30" spans="1:7" ht="150.75" x14ac:dyDescent="0.25">
-      <c r="A30" s="9"/>
+      <c r="A30" s="12"/>
       <c r="B30" s="4" t="s">
         <v>141</v>
       </c>
@@ -5159,11 +5453,11 @@
       <c r="E30" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="F30" s="7"/>
-      <c r="G30" s="7"/>
+      <c r="F30" s="13"/>
+      <c r="G30" s="13"/>
     </row>
     <row r="31" spans="1:7" ht="135.75" x14ac:dyDescent="0.25">
-      <c r="A31" s="9"/>
+      <c r="A31" s="12"/>
       <c r="B31" s="3" t="s">
         <v>145</v>
       </c>
@@ -5178,7 +5472,7 @@
       </c>
     </row>
     <row r="32" spans="1:7" ht="105.75" x14ac:dyDescent="0.25">
-      <c r="A32" s="9"/>
+      <c r="A32" s="12"/>
       <c r="B32" s="4" t="s">
         <v>149</v>
       </c>
@@ -5193,7 +5487,7 @@
       </c>
     </row>
     <row r="33" spans="1:18" ht="37.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A33" s="9" t="s">
+      <c r="A33" s="12" t="s">
         <v>152</v>
       </c>
       <c r="B33" s="5" t="s">
@@ -5216,7 +5510,7 @@
       </c>
     </row>
     <row r="34" spans="1:18" ht="172.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A34" s="9"/>
+      <c r="A34" s="12"/>
       <c r="B34" s="3" t="s">
         <v>159</v>
       </c>
@@ -5237,7 +5531,7 @@
       </c>
     </row>
     <row r="35" spans="1:18" ht="321" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A35" s="9"/>
+      <c r="A35" s="12"/>
       <c r="B35" s="3" t="s">
         <v>165</v>
       </c>
@@ -5258,7 +5552,7 @@
       </c>
     </row>
     <row r="36" spans="1:18" ht="198" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A36" s="9"/>
+      <c r="A36" s="12"/>
       <c r="B36" s="3" t="s">
         <v>172</v>
       </c>
@@ -5275,7 +5569,7 @@
       <c r="G36" s="3"/>
     </row>
     <row r="37" spans="1:18" ht="30" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A37" s="9" t="s">
+      <c r="A37" s="12" t="s">
         <v>176</v>
       </c>
       <c r="B37" s="5" t="s">
@@ -5289,7 +5583,7 @@
       </c>
     </row>
     <row r="38" spans="1:18" ht="212.25" x14ac:dyDescent="0.25">
-      <c r="A38" s="9"/>
+      <c r="A38" s="12"/>
       <c r="B38" s="3" t="s">
         <v>180</v>
       </c>
@@ -5301,63 +5595,63 @@
       </c>
     </row>
     <row r="39" spans="1:18" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A39" s="10" t="s">
+      <c r="A39" s="9" t="s">
         <v>64</v>
       </c>
       <c r="B39" s="5" t="s">
         <v>177</v>
       </c>
-      <c r="C39" s="8" t="s">
+      <c r="C39" s="7" t="s">
         <v>183</v>
       </c>
-      <c r="D39" s="8" t="s">
+      <c r="D39" s="7" t="s">
         <v>184</v>
       </c>
-      <c r="E39" s="8" t="s">
+      <c r="E39" s="7" t="s">
         <v>185</v>
       </c>
-      <c r="F39" s="8" t="s">
+      <c r="F39" s="7" t="s">
         <v>186</v>
       </c>
-      <c r="G39" s="8" t="s">
+      <c r="G39" s="7" t="s">
         <v>187</v>
       </c>
-      <c r="H39" s="8" t="s">
+      <c r="H39" s="7" t="s">
         <v>188</v>
       </c>
-      <c r="I39" s="8" t="s">
+      <c r="I39" s="7" t="s">
         <v>189</v>
       </c>
-      <c r="J39" s="8" t="s">
+      <c r="J39" s="7" t="s">
         <v>190</v>
       </c>
-      <c r="K39" s="8" t="s">
+      <c r="K39" s="7" t="s">
         <v>191</v>
       </c>
-      <c r="L39" s="8" t="s">
+      <c r="L39" s="7" t="s">
         <v>192</v>
       </c>
-      <c r="M39" s="8" t="s">
+      <c r="M39" s="7" t="s">
         <v>193</v>
       </c>
-      <c r="N39" s="8" t="s">
+      <c r="N39" s="7" t="s">
         <v>194</v>
       </c>
-      <c r="O39" s="8" t="s">
+      <c r="O39" s="7" t="s">
         <v>195</v>
       </c>
-      <c r="P39" s="8" t="s">
+      <c r="P39" s="7" t="s">
         <v>196</v>
       </c>
-      <c r="Q39" s="8" t="s">
+      <c r="Q39" s="7" t="s">
         <v>197</v>
       </c>
-      <c r="R39" s="8" t="s">
+      <c r="R39" s="7" t="s">
         <v>198</v>
       </c>
     </row>
     <row r="40" spans="1:18" ht="183.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A40" s="10"/>
+      <c r="A40" s="9"/>
       <c r="B40" s="3" t="s">
         <v>200</v>
       </c>
@@ -5411,7 +5705,7 @@
       </c>
     </row>
     <row r="41" spans="1:18" ht="300.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A41" s="10"/>
+      <c r="A41" s="9"/>
       <c r="B41" s="3" t="s">
         <v>218</v>
       </c>
@@ -5456,7 +5750,7 @@
       </c>
     </row>
     <row r="42" spans="1:18" ht="180.75" x14ac:dyDescent="0.25">
-      <c r="A42" s="10"/>
+      <c r="A42" s="9"/>
       <c r="B42" s="3"/>
       <c r="H42" s="3" t="s">
         <v>231</v>
@@ -5466,7 +5760,7 @@
       </c>
     </row>
     <row r="43" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A43" s="10" t="s">
+      <c r="A43" s="9" t="s">
         <v>89</v>
       </c>
       <c r="B43" s="5" t="s">
@@ -5486,7 +5780,7 @@
       </c>
     </row>
     <row r="44" spans="1:18" ht="135" x14ac:dyDescent="0.25">
-      <c r="A44" s="10"/>
+      <c r="A44" s="9"/>
       <c r="B44" s="3" t="s">
         <v>234</v>
       </c>
@@ -5504,7 +5798,7 @@
       </c>
     </row>
     <row r="45" spans="1:18" ht="270.75" x14ac:dyDescent="0.25">
-      <c r="A45" s="10"/>
+      <c r="A45" s="9"/>
       <c r="B45" s="3" t="s">
         <v>239</v>
       </c>
@@ -5522,13 +5816,13 @@
       </c>
     </row>
     <row r="46" spans="1:18" ht="290.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A46" s="10"/>
+      <c r="A46" s="9"/>
       <c r="E46" s="3" t="s">
         <v>244</v>
       </c>
     </row>
     <row r="47" spans="1:18" x14ac:dyDescent="0.25">
-      <c r="A47" s="10" t="s">
+      <c r="A47" s="9" t="s">
         <v>245</v>
       </c>
       <c r="B47" s="5" t="s">
@@ -5539,7 +5833,7 @@
       </c>
     </row>
     <row r="48" spans="1:18" ht="120" x14ac:dyDescent="0.25">
-      <c r="A48" s="10"/>
+      <c r="A48" s="9"/>
       <c r="B48" s="3" t="s">
         <v>248</v>
       </c>
@@ -5548,7 +5842,7 @@
       </c>
     </row>
     <row r="49" spans="1:7" ht="300.75" x14ac:dyDescent="0.25">
-      <c r="A49" s="10"/>
+      <c r="A49" s="9"/>
       <c r="B49" s="3" t="s">
         <v>250</v>
       </c>
@@ -5557,7 +5851,7 @@
       </c>
     </row>
     <row r="50" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A50" s="10" t="s">
+      <c r="A50" s="9" t="s">
         <v>252</v>
       </c>
       <c r="B50" s="5" t="s">
@@ -5580,7 +5874,7 @@
       </c>
     </row>
     <row r="51" spans="1:7" ht="165" x14ac:dyDescent="0.25">
-      <c r="A51" s="10"/>
+      <c r="A51" s="9"/>
       <c r="B51" s="3" t="s">
         <v>258</v>
       </c>
@@ -5601,7 +5895,7 @@
       </c>
     </row>
     <row r="52" spans="1:7" ht="346.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A52" s="10"/>
+      <c r="A52" s="9"/>
       <c r="B52" s="3" t="s">
         <v>264</v>
       </c>
@@ -5622,7 +5916,7 @@
       </c>
     </row>
     <row r="53" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A53" s="10" t="s">
+      <c r="A53" s="9" t="s">
         <v>270</v>
       </c>
       <c r="B53" s="5" t="s">
@@ -5639,7 +5933,7 @@
       </c>
     </row>
     <row r="54" spans="1:7" ht="159" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A54" s="10"/>
+      <c r="A54" s="9"/>
       <c r="B54" s="3" t="s">
         <v>274</v>
       </c>
@@ -5654,7 +5948,7 @@
       </c>
     </row>
     <row r="55" spans="1:7" ht="391.5" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A55" s="10"/>
+      <c r="A55" s="9"/>
       <c r="B55" s="3" t="s">
         <v>278</v>
       </c>
@@ -5669,7 +5963,7 @@
       </c>
     </row>
     <row r="56" spans="1:7" ht="225" x14ac:dyDescent="0.25">
-      <c r="A56" s="10"/>
+      <c r="A56" s="9"/>
       <c r="B56" s="3" t="s">
         <v>282</v>
       </c>
@@ -5684,7 +5978,7 @@
       </c>
     </row>
     <row r="57" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A57" s="11" t="s">
+      <c r="A57" s="10" t="s">
         <v>199</v>
       </c>
       <c r="B57" s="5" t="s">
@@ -5692,25 +5986,25 @@
       </c>
     </row>
     <row r="58" spans="1:7" ht="144.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A58" s="12"/>
+      <c r="A58" s="11"/>
       <c r="B58" s="3" t="s">
         <v>287</v>
       </c>
     </row>
-    <row r="59" spans="1:7" ht="209.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A59" s="12"/>
+    <row r="59" spans="1:7" ht="315.75" x14ac:dyDescent="0.25">
+      <c r="A59" s="11"/>
       <c r="B59" s="3" t="s">
+        <v>336</v>
+      </c>
+    </row>
+    <row r="60" spans="1:7" ht="135" x14ac:dyDescent="0.25">
+      <c r="A60" s="11"/>
+      <c r="B60" s="3" t="s">
         <v>288</v>
       </c>
     </row>
-    <row r="60" spans="1:7" ht="135" x14ac:dyDescent="0.25">
-      <c r="A60" s="12"/>
-      <c r="B60" s="3" t="s">
-        <v>289</v>
-      </c>
-    </row>
     <row r="61" spans="1:7" ht="27" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A61" s="9" t="s">
+      <c r="A61" s="12" t="s">
         <v>140</v>
       </c>
       <c r="B61" s="5" t="s">
@@ -5720,23 +6014,23 @@
         <v>178</v>
       </c>
       <c r="D61" s="5" t="s">
+        <v>289</v>
+      </c>
+    </row>
+    <row r="62" spans="1:7" ht="255.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A62" s="12"/>
+      <c r="B62" s="3" t="s">
         <v>290</v>
       </c>
-    </row>
-    <row r="62" spans="1:7" ht="255.75" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A62" s="9"/>
-      <c r="B62" s="3" t="s">
+      <c r="C62" s="3" t="s">
         <v>291</v>
       </c>
-      <c r="C62" s="3" t="s">
+      <c r="D62" s="3" t="s">
         <v>292</v>
       </c>
-      <c r="D62" s="3" t="s">
-        <v>293</v>
-      </c>
     </row>
     <row r="63" spans="1:7" x14ac:dyDescent="0.25">
-      <c r="A63" s="10" t="s">
+      <c r="A63" s="9" t="s">
         <v>144</v>
       </c>
       <c r="B63" s="5" t="s">
@@ -5746,23 +6040,23 @@
         <v>178</v>
       </c>
       <c r="D63" s="5" t="s">
+        <v>293</v>
+      </c>
+    </row>
+    <row r="64" spans="1:7" ht="165" x14ac:dyDescent="0.25">
+      <c r="A64" s="9"/>
+      <c r="B64" s="3" t="s">
         <v>294</v>
       </c>
-    </row>
-    <row r="64" spans="1:7" ht="165" x14ac:dyDescent="0.25">
-      <c r="A64" s="10"/>
-      <c r="B64" s="3" t="s">
+      <c r="C64" s="3" t="s">
         <v>295</v>
       </c>
-      <c r="C64" s="3" t="s">
+      <c r="D64" s="3" t="s">
         <v>296</v>
       </c>
-      <c r="D64" s="3" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
-      <c r="A65" s="10" t="s">
+    </row>
+    <row r="65" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A65" s="9" t="s">
         <v>148</v>
       </c>
       <c r="B65" s="5" t="s">
@@ -5772,17 +6066,203 @@
         <v>178</v>
       </c>
     </row>
-    <row r="66" spans="1:3" ht="236.25" customHeight="1" x14ac:dyDescent="0.25">
-      <c r="A66" s="10"/>
+    <row r="66" spans="1:9" ht="236.25" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A66" s="9"/>
       <c r="B66" s="3" t="s">
+        <v>297</v>
+      </c>
+      <c r="C66" s="3" t="s">
         <v>298</v>
       </c>
-      <c r="C66" s="3" t="s">
+    </row>
+    <row r="67" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A67" s="15" t="s">
         <v>299</v>
       </c>
+      <c r="B67" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C67" s="5" t="s">
+        <v>300</v>
+      </c>
+      <c r="D67" s="5" t="s">
+        <v>302</v>
+      </c>
+      <c r="E67" s="5" t="s">
+        <v>305</v>
+      </c>
+      <c r="F67" s="5" t="s">
+        <v>307</v>
+      </c>
+    </row>
+    <row r="68" spans="1:9" ht="150" x14ac:dyDescent="0.25">
+      <c r="A68" s="16"/>
+      <c r="B68" s="3" t="s">
+        <v>303</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>301</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>304</v>
+      </c>
+      <c r="E68" s="3" t="s">
+        <v>306</v>
+      </c>
+      <c r="F68" s="3" t="s">
+        <v>308</v>
+      </c>
+    </row>
+    <row r="69" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A69" s="15" t="s">
+        <v>316</v>
+      </c>
+      <c r="B69" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C69" s="5" t="s">
+        <v>310</v>
+      </c>
+      <c r="D69" s="5" t="s">
+        <v>312</v>
+      </c>
+      <c r="E69" s="5" t="s">
+        <v>315</v>
+      </c>
+    </row>
+    <row r="70" spans="1:9" ht="405" x14ac:dyDescent="0.25">
+      <c r="A70" s="16"/>
+      <c r="B70" s="3" t="s">
+        <v>309</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>311</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>313</v>
+      </c>
+      <c r="E70" s="3" t="s">
+        <v>314</v>
+      </c>
+    </row>
+    <row r="71" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A71" s="15" t="s">
+        <v>317</v>
+      </c>
+      <c r="B71" s="5" t="s">
+        <v>177</v>
+      </c>
+      <c r="C71" s="5" t="s">
+        <v>320</v>
+      </c>
+      <c r="D71" s="5" t="s">
+        <v>321</v>
+      </c>
+      <c r="E71" s="5" t="s">
+        <v>323</v>
+      </c>
+      <c r="F71" s="5" t="s">
+        <v>325</v>
+      </c>
+      <c r="G71" s="5" t="s">
+        <v>327</v>
+      </c>
+      <c r="H71" s="5" t="s">
+        <v>328</v>
+      </c>
+      <c r="I71" s="5" t="s">
+        <v>330</v>
+      </c>
+    </row>
+    <row r="72" spans="1:9" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A72" s="16"/>
+      <c r="B72" s="14" t="s">
+        <v>318</v>
+      </c>
+      <c r="C72" s="14" t="s">
+        <v>319</v>
+      </c>
+      <c r="D72" s="14" t="s">
+        <v>322</v>
+      </c>
+      <c r="E72" s="14" t="s">
+        <v>324</v>
+      </c>
+      <c r="F72" s="14" t="s">
+        <v>326</v>
+      </c>
+      <c r="G72" s="14" t="s">
+        <v>338</v>
+      </c>
+      <c r="H72" s="14" t="s">
+        <v>329</v>
+      </c>
+      <c r="I72" s="14" t="s">
+        <v>331</v>
+      </c>
+    </row>
+    <row r="74" spans="1:9" ht="18.75" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="A74" s="17" t="s">
+        <v>332</v>
+      </c>
+      <c r="B74" s="5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="75" spans="1:9" ht="409.5" x14ac:dyDescent="0.25">
+      <c r="A75" s="18"/>
+      <c r="B75" s="14" t="s">
+        <v>333</v>
+      </c>
+    </row>
+    <row r="76" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A76" s="17" t="s">
+        <v>334</v>
+      </c>
+      <c r="B76" s="5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="77" spans="1:9" ht="135" x14ac:dyDescent="0.25">
+      <c r="A77" s="18"/>
+      <c r="B77" s="14" t="s">
+        <v>335</v>
+      </c>
+    </row>
+    <row r="78" spans="1:9" x14ac:dyDescent="0.25">
+      <c r="A78" s="15" t="s">
+        <v>337</v>
+      </c>
+      <c r="B78" s="5" t="s">
+        <v>177</v>
+      </c>
+    </row>
+    <row r="79" spans="1:9" ht="210" x14ac:dyDescent="0.25">
+      <c r="A79" s="16"/>
+      <c r="B79" s="14" t="s">
+        <v>339</v>
+      </c>
     </row>
   </sheetData>
-  <mergeCells count="20">
+  <mergeCells count="26">
+    <mergeCell ref="A78:A79"/>
+    <mergeCell ref="A67:A68"/>
+    <mergeCell ref="A69:A70"/>
+    <mergeCell ref="A71:A72"/>
+    <mergeCell ref="A74:A75"/>
+    <mergeCell ref="A76:A77"/>
+    <mergeCell ref="A39:A42"/>
+    <mergeCell ref="A1:A5"/>
+    <mergeCell ref="A6:A9"/>
+    <mergeCell ref="A10:A13"/>
+    <mergeCell ref="A14:A18"/>
+    <mergeCell ref="A19:A22"/>
+    <mergeCell ref="A23:A26"/>
+    <mergeCell ref="A27:A32"/>
+    <mergeCell ref="F29:F30"/>
+    <mergeCell ref="G29:G30"/>
+    <mergeCell ref="A33:A36"/>
+    <mergeCell ref="A37:A38"/>
     <mergeCell ref="A63:A64"/>
     <mergeCell ref="A65:A66"/>
     <mergeCell ref="A43:A46"/>
@@ -5791,18 +6271,6 @@
     <mergeCell ref="A53:A56"/>
     <mergeCell ref="A57:A60"/>
     <mergeCell ref="A61:A62"/>
-    <mergeCell ref="A27:A32"/>
-    <mergeCell ref="F29:F30"/>
-    <mergeCell ref="G29:G30"/>
-    <mergeCell ref="A33:A36"/>
-    <mergeCell ref="A37:A38"/>
-    <mergeCell ref="A39:A42"/>
-    <mergeCell ref="A1:A5"/>
-    <mergeCell ref="A6:A9"/>
-    <mergeCell ref="A10:A13"/>
-    <mergeCell ref="A14:A18"/>
-    <mergeCell ref="A19:A22"/>
-    <mergeCell ref="A23:A26"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>